<commit_message>
added color scheme for victims and tiles
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meine Ablage\HTL-Google Drive\PROJEKTE\ROBOTIK\ROBOCUP JUNIOR 2026\robotics_framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF15F1DD-3537-4AFF-9B40-99D85609B19B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CFA26B-153B-4D19-9E52-1BA4716B073D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C010B32C-7C53-4A6E-B683-211E5868A042}"/>
   </bookViews>
@@ -39,10 +39,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
-    <t>S</t>
+    <t>X</t>
   </si>
   <si>
-    <t>X</t>
+    <t>SW</t>
   </si>
 </sst>
 </file>
@@ -146,9 +146,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -158,10 +155,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -173,6 +173,7 @@
   <colors>
     <mruColors>
       <color rgb="FF0000FF"/>
+      <color rgb="FF00FFFF"/>
     </mruColors>
   </colors>
   <extLst>
@@ -184,6 +185,195 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>320566</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>204950</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>120869</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>478219</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Textfeld 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{181FD914-5656-4874-9A53-06736C2E2F55}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3946635" y="204950"/>
+          <a:ext cx="3426372" cy="3804745"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>Color Victims:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>ROT =&gt; roter Rand (255,0,0)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>GELB =&gt; gelber Rand (255,255,0)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>GRÜN =&gt; grüner Rand (0,255,0)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>Letter Victims:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>H =&gt; blauer Rand (0,0,255)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>S =&gt; türkiser Rand (0,255,255)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>U =&gt;lila Rand (255,0,255)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="de-AT" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>Colored Tiles:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>WEISS (255,255,255) =&gt; None</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>ROT (255,0,0) =&gt; Eingang in Gefahrenzone</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>SCHARZ (0,0,0)=&gt; Loch (vermeiden)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>SILBER/GRAU (128,128,128) =&gt; Checkpoints</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>BLAU (0,0,255) =&gt; schwer begebar (5sec wait)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="de-AT" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>START Tile:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>SW =&gt; Robter nach Westen ausgrichtet</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>SO =&gt; Roboter nach Osten ausgerichtet</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>SS =&gt; Roboter nach Süden ausgerichtet</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>SN oder S =&gt; Roboter nach Norden ausgerichtet</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -486,28 +676,31 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="8.77734375" style="1"/>
+    <col min="1" max="6" width="8.77734375" style="1"/>
+    <col min="7" max="7" width="8.77734375" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="40.049999999999997" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="5"/>
+      <c r="A1" s="5"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="4"/>
     </row>
     <row r="2" spans="1:4" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="3"/>
+      <c r="A2" s="6"/>
+      <c r="B2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:4" ht="40.049999999999997" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="D3" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="1200" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
improved victim settings added victim letter display and recognition
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meine Ablage\HTL-Google Drive\PROJEKTE\ROBOTIK\ROBOCUP JUNIOR 2026\robotics_framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CFA26B-153B-4D19-9E52-1BA4716B073D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F407E30-A4F4-4E1F-8A5F-E5B866AD1BAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C010B32C-7C53-4A6E-B683-211E5868A042}"/>
   </bookViews>
@@ -72,7 +72,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -132,9 +132,22 @@
         <color auto="1"/>
       </right>
       <top style="thick">
-        <color rgb="FFFF0000"/>
+        <color auto="1"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -146,22 +159,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -199,8 +212,8 @@
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>120869</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>478219</xdr:rowOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>136634</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -216,7 +229,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3946635" y="204950"/>
-          <a:ext cx="3426372" cy="3804745"/>
+          <a:ext cx="3426372" cy="4976650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -252,8 +265,42 @@
         <a:p>
           <a:r>
             <a:rPr lang="de-AT" sz="1100"/>
-            <a:t>Color Victims:</a:t>
-          </a:r>
+            <a:t>COLOR</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100" baseline="0"/>
+            <a:t> VICTIMS:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100" baseline="0"/>
+            <a:t>Codes example:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100" baseline="0"/>
+            <a:t>VCRE =&gt; VC (victim color), R (color red), E (wall east)</a:t>
+          </a:r>
+          <a:endParaRPr lang="de-AT" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>Farben:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100" baseline="0"/>
+            <a:t> red, yellow, green</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100" baseline="0"/>
+            <a:t>Richtung der Wand: n, e, s, w</a:t>
+          </a:r>
+          <a:endParaRPr lang="de-AT" sz="1100"/>
         </a:p>
         <a:p>
           <a:r>
@@ -274,10 +321,55 @@
           </a:r>
         </a:p>
         <a:p>
-          <a:r>
-            <a:rPr lang="de-AT" sz="1100"/>
-            <a:t>Letter Victims:</a:t>
-          </a:r>
+          <a:endParaRPr lang="de-AT" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>LETTER</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100" baseline="0"/>
+            <a:t> VICTIMS</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Codes example:</a:t>
+          </a:r>
+          <a:endParaRPr lang="de-AT">
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>VLHW =&gt; VL (victim letter), H (letter), w (wall west)</a:t>
+          </a:r>
+          <a:endParaRPr lang="de-AT">
+            <a:effectLst/>
+          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:r>
@@ -303,7 +395,15 @@
         <a:p>
           <a:r>
             <a:rPr lang="de-AT" sz="1100"/>
-            <a:t>Colored Tiles:</a:t>
+            <a:t>COLORED</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100" baseline="0"/>
+            <a:t> TILES</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="de-AT" sz="1100"/>
+            <a:t>:</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -342,7 +442,7 @@
         <a:p>
           <a:r>
             <a:rPr lang="de-AT" sz="1100"/>
-            <a:t>START Tile:</a:t>
+            <a:t>START TILE:</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -682,16 +782,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="40.049999999999997" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5"/>
-      <c r="B1" s="3"/>
-      <c r="C1" s="4"/>
+      <c r="A1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="3"/>
     </row>
     <row r="2" spans="1:4" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="6"/>
-      <c r="B2" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="7"/>
     </row>
     <row r="3" spans="1:4" ht="40.049999999999997" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="D3" s="1" t="s">

</xml_diff>